<commit_message>
Add section-wise exam question selection , AI generated Question and update exam application
</commit_message>
<xml_diff>
--- a/backend/static/DB.xlsx
+++ b/backend/static/DB.xlsx
@@ -425,7 +425,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Databricks Fundamentals</t>
+          <t>Placement Test</t>
         </is>
       </c>
     </row>
@@ -484,8 +484,11 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G11"/>
+  <dimension ref="A1:H11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="20" customWidth="1" min="8" max="8"/>
+  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
@@ -523,6 +526,11 @@
           <t>Correct Answer</t>
         </is>
       </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>Section</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="n">
@@ -530,32 +538,37 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>What is Databricks primarily used for?</t>
+          <t>A train 120 m long passes a pole in 6 seconds. What is its speed?</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Data Analytics and AI</t>
+          <t>10 m/s</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Web Development</t>
+          <t>15 m/s</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>Mobile Development</t>
+          <t>20 m/s</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>Game Development</t>
+          <t>25 m/s</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>Aptitude</t>
         </is>
       </c>
     </row>
@@ -565,32 +578,37 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Which processing engine is used by Databricks?</t>
+          <t>What is 20% of 250?</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Hadoop</t>
+          <t>25</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Spark</t>
+          <t>40</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>Tomcat</t>
+          <t>50</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>Nginx</t>
+          <t>75</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>Aptitude</t>
         </is>
       </c>
     </row>
@@ -600,32 +618,37 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Which language is NOT supported by Databricks notebooks?</t>
+          <t>Find the next number: 2, 6, 12, 20, ?</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Python</t>
+          <t>28</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>SQL</t>
+          <t>30</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>Scala</t>
+          <t>32</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>PHP</t>
+          <t>36</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>Reasoning</t>
         </is>
       </c>
     </row>
@@ -635,32 +658,37 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>What is DBFS in Databricks?</t>
+          <t>If CAT is coded as DBU, how is DOG coded?</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Database File System</t>
+          <t>EPH</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>Distributed Backup File System</t>
+          <t>EPI</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>Data Backup Feature Service</t>
+          <t>FPH</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>Database Format Service</t>
+          <t>DPH</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
           <t>A</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>Reasoning</t>
         </is>
       </c>
     </row>
@@ -670,32 +698,37 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Which cloud platforms support Databricks?</t>
+          <t>Choose the correct sentence.</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>AWS</t>
+          <t>She do not like tea.</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>Azure</t>
+          <t>She does not likes tea.</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>Google Cloud</t>
+          <t>She does not like tea.</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>All of the Above</t>
+          <t>She not like tea.</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>English Grammar</t>
         </is>
       </c>
     </row>
@@ -705,175 +738,44 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>What is a Databricks Cluster?</t>
+          <t>Fill in the blank: He has been working here ___ 2019.</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>A Group of Servers for Processing</t>
+          <t>for</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>A Database Table</t>
+          <t>since</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>A Programming Language</t>
+          <t>from</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>A Dashboard</t>
+          <t>at</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>A</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="n">
-        <v>7</v>
-      </c>
-      <c r="B8" t="inlineStr">
-        <is>
-          <t>Which command displays the contents of DBFS?</t>
-        </is>
-      </c>
-      <c r="C8" t="inlineStr">
-        <is>
-          <t>%fs ls</t>
-        </is>
-      </c>
-      <c r="D8" t="inlineStr">
-        <is>
-          <t>%db ls</t>
-        </is>
-      </c>
-      <c r="E8" t="inlineStr">
-        <is>
-          <t>%list fs</t>
-        </is>
-      </c>
-      <c r="F8" t="inlineStr">
-        <is>
-          <t>%show dbfs</t>
-        </is>
-      </c>
-      <c r="G8" t="inlineStr">
-        <is>
-          <t>A</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="n">
-        <v>8</v>
-      </c>
-      <c r="B9" t="inlineStr">
-        <is>
-          <t>What is Delta Lake in Databricks?</t>
-        </is>
-      </c>
-      <c r="C9" t="inlineStr">
-        <is>
-          <t>Storage Layer</t>
-        </is>
-      </c>
-      <c r="D9" t="inlineStr">
-        <is>
-          <t>UI Framework</t>
-        </is>
-      </c>
-      <c r="E9" t="inlineStr">
-        <is>
-          <t>Web Server</t>
-        </is>
-      </c>
-      <c r="F9" t="inlineStr">
-        <is>
-          <t>Deployment Tool</t>
-        </is>
-      </c>
-      <c r="G9" t="inlineStr">
-        <is>
-          <t>A</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="n">
-        <v>9</v>
-      </c>
-      <c r="B10" t="inlineStr">
-        <is>
-          <t>Which notebook language magic command is used for Python?</t>
-        </is>
-      </c>
-      <c r="C10" t="inlineStr">
-        <is>
-          <t>%py</t>
-        </is>
-      </c>
-      <c r="D10" t="inlineStr">
-        <is>
-          <t>%python</t>
-        </is>
-      </c>
-      <c r="E10" t="inlineStr">
-        <is>
-          <t>%p</t>
-        </is>
-      </c>
-      <c r="F10" t="inlineStr">
-        <is>
-          <t>%code</t>
-        </is>
-      </c>
-      <c r="G10" t="inlineStr">
-        <is>
           <t>B</t>
         </is>
       </c>
-    </row>
-    <row r="11">
-      <c r="A11" t="n">
-        <v>10</v>
-      </c>
-      <c r="B11" t="inlineStr">
-        <is>
-          <t>What is the purpose of a Databricks Workspace?</t>
-        </is>
-      </c>
-      <c r="C11" t="inlineStr">
-        <is>
-          <t>To Manage Notebooks and Resources</t>
-        </is>
-      </c>
-      <c r="D11" t="inlineStr">
-        <is>
-          <t>To Host Websites</t>
-        </is>
-      </c>
-      <c r="E11" t="inlineStr">
-        <is>
-          <t>To Store Images</t>
-        </is>
-      </c>
-      <c r="F11" t="inlineStr">
-        <is>
-          <t>To Configure Routers</t>
-        </is>
-      </c>
-      <c r="G11" t="inlineStr">
-        <is>
-          <t>A</t>
-        </is>
-      </c>
-    </row>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>English Grammar</t>
+        </is>
+      </c>
+    </row>
+    <row r="8"/>
+    <row r="9"/>
+    <row r="10"/>
+    <row r="11"/>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>